<commit_message>
Fix heading hierarchy for accessibility + footer label
- wknd-cleanup transformer: normalize non-structural headings (byline,
  "SHARE THIS STORY", duplicate title) so document outline is monotonic
- footer "Follow Us" h5 -> styled paragraph
- re-import magazine pages with normalized headings

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-magazine.report.xlsx
+++ b/tools/importer/reports/import-magazine.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="152">
   <si>
     <t>_reportFile</t>
   </si>
@@ -61,6 +61,27 @@
     <t>https://wknd.site/us/en.html</t>
   </si>
   <si>
+    <t>us/en/about-us.report.json</t>
+  </si>
+  <si>
+    <t>["writer-details-xf","writer-details-xf","writer-details-xf","writer-details-xf","writer-details-xf","writer-details-xf","writer-details-xf"]</t>
+  </si>
+  <si>
+    <t>us/en/about-us</t>
+  </si>
+  <si>
+    <t>about-us</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:30:00.812Z</t>
+  </si>
+  <si>
+    <t>About Us</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/about-us.html</t>
+  </si>
+  <si>
     <t>us/en/adventures.report.json</t>
   </si>
   <si>
@@ -82,6 +103,291 @@
     <t>https://wknd.site/us/en/adventures.html</t>
   </si>
   <si>
+    <t>us/en/faqs.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq"]</t>
+  </si>
+  <si>
+    <t>us/en/faqs</t>
+  </si>
+  <si>
+    <t>faqs</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:36:48.470Z</t>
+  </si>
+  <si>
+    <t>FAQs</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/faqs.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine.report.json</t>
+  </si>
+  <si>
+    <t>["columns-featured","cards-article"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:30:07.056Z</t>
+  </si>
+  <si>
+    <t>Magazine</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>["carousel-gallery","columns-details","social-links","tabs-content"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>adventures</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:19:34.798Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:19:40.050Z</t>
+  </si>
+  <si>
+    <t>Beervana in Portland</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:19:44.938Z</t>
+  </si>
+  <si>
+    <t>Climbing New Zealand</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:19:49.139Z</t>
+  </si>
+  <si>
+    <t>Colorado Rock Climbing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/colorado-rock-climbing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:19:53.394Z</t>
+  </si>
+  <si>
+    <t>Cycling Southern Utah</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:19:58.011Z</t>
+  </si>
+  <si>
+    <t>Cycling Tuscany</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-tuscany.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:20:01.919Z</t>
+  </si>
+  <si>
+    <t>Downhill Skiing Wyoming</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/downhill-skiing-wyoming.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:20:06.041Z</t>
+  </si>
+  <si>
+    <t>Gastronomic Marais Tour</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/gastronomic-marais-tour.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:20:11.631Z</t>
+  </si>
+  <si>
+    <t>Napa Wine Tasting</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/napa-wine-tasting.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:20:16.794Z</t>
+  </si>
+  <si>
+    <t>Riverside Camping</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/riverside-camping-australia.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:20:22.659Z</t>
+  </si>
+  <si>
+    <t>Ski Touring Mont Blanc</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/ski-touring-mont-blanc.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:20:26.971Z</t>
+  </si>
+  <si>
+    <t>Surf Camp in Costa Rica</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/surf-camp-costa-rica.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:20:31.968Z</t>
+  </si>
+  <si>
+    <t>Tahoe Skiing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:20:36.213Z</t>
+  </si>
+  <si>
+    <t>West Coast Cycling</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/west-coast-cycling.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:20:40.540Z</t>
+  </si>
+  <si>
+    <t>Whistler Mountain Biking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/whistler-mountain-biking.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-09-08T16:20:45.029Z</t>
+  </si>
+  <si>
+    <t>Yosemite Backpacking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
+  </si>
+  <si>
     <t>us/en/magazine/arctic-surfing.report.json</t>
   </si>
   <si>
@@ -94,7 +400,7 @@
     <t>magazine</t>
   </si>
   <si>
-    <t>2026-09-08T16:03:33.135Z</t>
+    <t>2026-09-08T18:50:22.625Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -109,7 +415,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-08T16:03:38.509Z</t>
+    <t>2026-09-08T18:50:28.261Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -124,7 +430,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-08T16:03:45.090Z</t>
+    <t>2026-09-08T18:50:33.365Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -139,7 +445,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-08T16:03:51.097Z</t>
+    <t>2026-09-08T18:50:38.510Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -154,7 +460,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-08T16:03:56.251Z</t>
+    <t>2026-09-08T18:50:44.728Z</t>
   </si>
   <si>
     <t>Western Australia</t>
@@ -549,12 +855,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="48" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="46" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="33" customWidth="1"/>
@@ -670,103 +975,597 @@
         <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="F7" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="G7" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="H7" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
         <v>46</v>
       </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>26</v>
-      </c>
       <c r="F8" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="G8" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="H8" t="s">
-        <v>49</v>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" t="s">
+        <v>63</v>
+      </c>
+      <c r="H10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" t="s">
+        <v>78</v>
+      </c>
+      <c r="H13" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" t="s">
+        <v>82</v>
+      </c>
+      <c r="G14" t="s">
+        <v>83</v>
+      </c>
+      <c r="H14" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" t="s">
+        <v>86</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" t="s">
+        <v>88</v>
+      </c>
+      <c r="H15" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" t="s">
+        <v>91</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" t="s">
+        <v>92</v>
+      </c>
+      <c r="G16" t="s">
+        <v>93</v>
+      </c>
+      <c r="H16" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" t="s">
+        <v>97</v>
+      </c>
+      <c r="G17" t="s">
+        <v>98</v>
+      </c>
+      <c r="H17" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>100</v>
+      </c>
+      <c r="B18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" t="s">
+        <v>101</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>46</v>
+      </c>
+      <c r="F18" t="s">
+        <v>102</v>
+      </c>
+      <c r="G18" t="s">
+        <v>103</v>
+      </c>
+      <c r="H18" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" t="s">
+        <v>106</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" t="s">
+        <v>107</v>
+      </c>
+      <c r="G19" t="s">
+        <v>108</v>
+      </c>
+      <c r="H19" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>110</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s">
+        <v>111</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" t="s">
+        <v>112</v>
+      </c>
+      <c r="G20" t="s">
+        <v>113</v>
+      </c>
+      <c r="H20" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>115</v>
+      </c>
+      <c r="B21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" t="s">
+        <v>116</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" t="s">
+        <v>117</v>
+      </c>
+      <c r="G21" t="s">
+        <v>118</v>
+      </c>
+      <c r="H21" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" t="s">
+        <v>121</v>
+      </c>
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>46</v>
+      </c>
+      <c r="F22" t="s">
+        <v>122</v>
+      </c>
+      <c r="G22" t="s">
+        <v>123</v>
+      </c>
+      <c r="H22" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" t="s">
+        <v>126</v>
+      </c>
+      <c r="C23" t="s">
+        <v>127</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>128</v>
+      </c>
+      <c r="F23" t="s">
+        <v>129</v>
+      </c>
+      <c r="G23" t="s">
+        <v>130</v>
+      </c>
+      <c r="H23" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>132</v>
+      </c>
+      <c r="B24" t="s">
+        <v>126</v>
+      </c>
+      <c r="C24" t="s">
+        <v>133</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>128</v>
+      </c>
+      <c r="F24" t="s">
+        <v>134</v>
+      </c>
+      <c r="G24" t="s">
+        <v>135</v>
+      </c>
+      <c r="H24" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>137</v>
+      </c>
+      <c r="B25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" t="s">
+        <v>138</v>
+      </c>
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>128</v>
+      </c>
+      <c r="F25" t="s">
+        <v>139</v>
+      </c>
+      <c r="G25" t="s">
+        <v>140</v>
+      </c>
+      <c r="H25" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>142</v>
+      </c>
+      <c r="B26" t="s">
+        <v>126</v>
+      </c>
+      <c r="C26" t="s">
+        <v>143</v>
+      </c>
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
+        <v>128</v>
+      </c>
+      <c r="F26" t="s">
+        <v>144</v>
+      </c>
+      <c r="G26" t="s">
+        <v>145</v>
+      </c>
+      <c r="H26" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>147</v>
+      </c>
+      <c r="B27" t="s">
+        <v>126</v>
+      </c>
+      <c r="C27" t="s">
+        <v>148</v>
+      </c>
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>128</v>
+      </c>
+      <c r="F27" t="s">
+        <v>149</v>
+      </c>
+      <c r="G27" t="s">
+        <v>150</v>
+      </c>
+      <c r="H27" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>